<commit_message>
Add measured max-Sinkhorn sheet from real emulator kernel runs
measure_kernels.py runs the matmul inner loop, softmax.asm, sinkhorn_iter.asm
and sinkhorn_col.asm in the wide-FP32 emulator and extracts measured cycle
rates (matmul 3 cyc/MAC-step + 6/tile, softmax 19/128-row, Sinkhorn row 9.1/row,
col 16.3/row). add_measured_sheet.py scales these to the SuperGlue op sizes and
writes "SG max-Sinkhorn (measured)": 418.5k us -> 2.39 FPS (vs 3.70 analytical;
the rolled matmul loop costs 3 cyc/MAC vs the bare-op count of 2). Matmul is
~98%; max-Sinkhorn itself is 6.5M of 418M cycles (1.5%).

https://claude.ai/code/session_01Wj1AhpfDtCg3YHVUGoUUbF
</commit_message>
<xml_diff>
--- a/IPU_2_SuperGlue.xlsx
+++ b/IPU_2_SuperGlue.xlsx
@@ -12,6 +12,7 @@
     <sheet name="SG base2-softmax" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="SG transpose-free col" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="SG fixed-thresh match" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SG max-Sinkhorn (measured)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -11358,6 +11359,7 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
+      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -11444,6 +11446,7 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
+      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -11530,6 +11533,7 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
+      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -11616,6 +11620,7 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
+      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -11702,6 +11707,7 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
+      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -11788,6 +11794,7 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
+      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -11874,6 +11881,7 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
+      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -11969,6 +11977,7 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
+      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -12146,6 +12155,7 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
+      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -12232,6 +12242,7 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
+      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -12318,6 +12329,7 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
+      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -12404,6 +12416,7 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
+      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -12490,6 +12503,7 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
+      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -12572,6 +12586,7 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -12654,6 +12669,7 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -12736,6 +12752,7 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -12822,6 +12839,7 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
+      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -12908,6 +12926,7 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
+      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -12994,6 +13013,7 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
+      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -13080,6 +13100,7 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
+      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -13166,6 +13187,7 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
+      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -13252,6 +13274,7 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
+      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -13338,6 +13361,7 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
+      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -13424,6 +13448,7 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
+      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -13510,6 +13535,7 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
+      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -13596,6 +13622,7 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
+      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -13687,6 +13714,7 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
+      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -13773,6 +13801,7 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
+      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -13859,6 +13888,7 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
+      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -13945,6 +13975,7 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
+      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -14031,6 +14062,7 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
+      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -14117,6 +14149,7 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
+      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -14203,6 +14236,7 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
+      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -14289,6 +14323,7 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
+      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -14375,6 +14410,7 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
+      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -14470,6 +14506,7 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
+      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -14647,6 +14684,7 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
+      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -14733,6 +14771,7 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
+      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -14819,6 +14858,7 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
+      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -14905,6 +14945,7 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
+      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -14987,6 +15028,7 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -15073,6 +15115,7 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
+      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -15159,6 +15202,7 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
+      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -15245,6 +15289,7 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
+      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -15331,6 +15376,7 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
+      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -15417,6 +15463,7 @@
         <f>((R51*8*1024)/$T51)/1000</f>
         <v/>
       </c>
+      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -15503,6 +15550,7 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
+      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -15589,6 +15637,7 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
+      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -15675,6 +15724,7 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
+      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -15761,6 +15811,7 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
+      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -15847,6 +15898,7 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
+      <c r="AA56" s="47" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -15942,6 +15994,7 @@
         <f>100*(SUM(T47:T57))</f>
         <v/>
       </c>
+      <c r="AA57" s="47" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -16028,6 +16081,7 @@
         <f>((R58*8*1024)/$T58)/1000</f>
         <v/>
       </c>
+      <c r="AA58" s="47" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -16114,6 +16168,7 @@
         <f>((R59*8*1024)/$T59)/1000</f>
         <v/>
       </c>
+      <c r="AA59" s="47" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -16200,6 +16255,7 @@
         <f>((R60*8*1024)/$T60)/1000</f>
         <v/>
       </c>
+      <c r="AA60" s="47" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -16286,6 +16342,7 @@
         <f>((R61*8*1024)/$T61)/1000</f>
         <v/>
       </c>
+      <c r="AA61" s="47" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -16372,6 +16429,7 @@
         <f>((R62*8*1024)/$T62)/1000</f>
         <v/>
       </c>
+      <c r="AA62" s="48" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -16850,6 +16908,7 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
+      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -16936,6 +16995,7 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
+      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -17022,6 +17082,7 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
+      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -17108,6 +17169,7 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
+      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -17194,6 +17256,7 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
+      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -17280,6 +17343,7 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
+      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -17366,6 +17430,7 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
+      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -17461,6 +17526,7 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
+      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -17638,6 +17704,7 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
+      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -17724,6 +17791,7 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
+      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -17810,6 +17878,7 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
+      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -17896,6 +17965,7 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
+      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -17982,6 +18052,7 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
+      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -18064,6 +18135,7 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -18146,6 +18218,7 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -18228,6 +18301,7 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -18314,6 +18388,7 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
+      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -18400,6 +18475,7 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
+      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -18486,6 +18562,7 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
+      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -18572,6 +18649,7 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
+      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -18658,6 +18736,7 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
+      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -18744,6 +18823,7 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
+      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -18830,6 +18910,7 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
+      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -18916,6 +18997,7 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
+      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -19002,6 +19084,7 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
+      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -19088,6 +19171,7 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
+      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -19179,6 +19263,7 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
+      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -19265,6 +19350,7 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
+      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -19351,6 +19437,7 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
+      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -19437,6 +19524,7 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
+      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -19523,6 +19611,7 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
+      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -19609,6 +19698,7 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
+      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -19695,6 +19785,7 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
+      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -19781,6 +19872,7 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
+      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -19867,6 +19959,7 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
+      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -19962,6 +20055,7 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
+      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -20139,6 +20233,7 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
+      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -20225,6 +20320,7 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
+      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -20311,6 +20407,7 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
+      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -20397,6 +20494,7 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
+      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -20479,6 +20577,7 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -20565,6 +20664,7 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
+      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -20651,6 +20751,7 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
+      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -20737,6 +20838,7 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
+      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -20823,6 +20925,7 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
+      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -20918,6 +21021,7 @@
         <f>100*(SUM(T47:T51))</f>
         <v/>
       </c>
+      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -21004,6 +21108,7 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
+      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -21090,6 +21195,7 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
+      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -21176,6 +21282,7 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
+      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -21262,6 +21369,7 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
+      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -21348,6 +21456,7 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
+      <c r="AA56" s="48" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -21826,6 +21935,7 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
+      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -21912,6 +22022,7 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
+      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -21998,6 +22109,7 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
+      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -22084,6 +22196,7 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
+      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -22170,6 +22283,7 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
+      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -22256,6 +22370,7 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
+      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -22342,6 +22457,7 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
+      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -22437,6 +22553,7 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
+      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -22614,6 +22731,7 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
+      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -22700,6 +22818,7 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
+      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -22786,6 +22905,7 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
+      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -22872,6 +22992,7 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
+      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -22958,6 +23079,7 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
+      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -23040,6 +23162,7 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -23122,6 +23245,7 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -23204,6 +23328,7 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -23290,6 +23415,7 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
+      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -23376,6 +23502,7 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
+      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -23462,6 +23589,7 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
+      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -23548,6 +23676,7 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
+      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -23634,6 +23763,7 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
+      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -23720,6 +23850,7 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
+      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -23806,6 +23937,7 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
+      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -23892,6 +24024,7 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
+      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -23978,6 +24111,7 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
+      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -24064,6 +24198,7 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
+      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -24155,6 +24290,7 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
+      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -24241,6 +24377,7 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
+      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -24327,6 +24464,7 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
+      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -24413,6 +24551,7 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
+      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -24499,6 +24638,7 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
+      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -24585,6 +24725,7 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
+      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -24671,6 +24812,7 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
+      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -24757,6 +24899,7 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
+      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -24843,6 +24986,7 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
+      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -24938,6 +25082,7 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
+      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -25115,6 +25260,7 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
+      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -25201,6 +25347,7 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
+      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -25287,6 +25434,7 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
+      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -25373,6 +25521,7 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
+      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -25455,6 +25604,7 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -25541,6 +25691,7 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
+      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -25627,6 +25778,7 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
+      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -25713,6 +25865,7 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
+      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -25799,6 +25952,7 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
+      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -25885,6 +26039,7 @@
         <f>((R51*8*1024)/$T51)/1000</f>
         <v/>
       </c>
+      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -25971,6 +26126,7 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
+      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -26057,6 +26213,7 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
+      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -26143,6 +26300,7 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
+      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -26229,6 +26387,7 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
+      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -26315,6 +26474,7 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
+      <c r="AA56" s="47" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -26410,6 +26570,7 @@
         <f>100*(SUM(T47:T57))</f>
         <v/>
       </c>
+      <c r="AA57" s="47" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -26496,6 +26657,7 @@
         <f>((R58*8*1024)/$T58)/1000</f>
         <v/>
       </c>
+      <c r="AA58" s="47" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -26582,6 +26744,7 @@
         <f>((R59*8*1024)/$T59)/1000</f>
         <v/>
       </c>
+      <c r="AA59" s="47" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -26668,6 +26831,7 @@
         <f>((R60*8*1024)/$T60)/1000</f>
         <v/>
       </c>
+      <c r="AA60" s="47" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -26754,6 +26918,7 @@
         <f>((R61*8*1024)/$T61)/1000</f>
         <v/>
       </c>
+      <c r="AA61" s="47" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -26840,6 +27005,7 @@
         <f>((R62*8*1024)/$T62)/1000</f>
         <v/>
       </c>
+      <c r="AA62" s="48" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -27318,6 +27484,7 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
+      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -27404,6 +27571,7 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
+      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -27490,6 +27658,7 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
+      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -27576,6 +27745,7 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
+      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -27662,6 +27832,7 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
+      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -27748,6 +27919,7 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
+      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -27834,6 +28006,7 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
+      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -27929,6 +28102,7 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
+      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -28106,6 +28280,7 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
+      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -28192,6 +28367,7 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
+      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -28278,6 +28454,7 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
+      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -28364,6 +28541,7 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
+      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -28450,6 +28628,7 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
+      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -28532,6 +28711,7 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -28614,6 +28794,7 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -28696,6 +28877,7 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -28782,6 +28964,7 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
+      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -28868,6 +29051,7 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
+      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -28954,6 +29138,7 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
+      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -29040,6 +29225,7 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
+      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -29126,6 +29312,7 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
+      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -29212,6 +29399,7 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
+      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -29298,6 +29486,7 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
+      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -29384,6 +29573,7 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
+      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -29470,6 +29660,7 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
+      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -29556,6 +29747,7 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
+      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -29647,6 +29839,7 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
+      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -29733,6 +29926,7 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
+      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -29819,6 +30013,7 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
+      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -29905,6 +30100,7 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
+      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -29991,6 +30187,7 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
+      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -30077,6 +30274,7 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
+      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -30163,6 +30361,7 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
+      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -30249,6 +30448,7 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
+      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -30335,6 +30535,7 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
+      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -30430,6 +30631,7 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
+      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -30607,6 +30809,7 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
+      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -30693,6 +30896,7 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
+      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -30779,6 +30983,7 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
+      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -30865,6 +31070,7 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
+      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -30947,6 +31153,7 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -31033,6 +31240,7 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
+      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -31119,6 +31327,7 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
+      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -31205,6 +31414,7 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
+      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -31291,6 +31501,7 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
+      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -31377,6 +31588,7 @@
         <f>((R51*8*1024)/$T51)/1000</f>
         <v/>
       </c>
+      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -31463,6 +31675,7 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
+      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -31549,6 +31762,7 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
+      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -31635,6 +31849,7 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
+      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -31721,6 +31936,7 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
+      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -31816,6 +32032,7 @@
         <f>100*(SUM(T47:T56))</f>
         <v/>
       </c>
+      <c r="AA56" s="47" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -31902,6 +32119,7 @@
         <f>((R57*8*1024)/$T57)/1000</f>
         <v/>
       </c>
+      <c r="AA57" s="47" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -31988,6 +32206,7 @@
         <f>((R58*8*1024)/$T58)/1000</f>
         <v/>
       </c>
+      <c r="AA58" s="47" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -32074,6 +32293,7 @@
         <f>((R59*8*1024)/$T59)/1000</f>
         <v/>
       </c>
+      <c r="AA59" s="47" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -32160,6 +32380,7 @@
         <f>((R60*8*1024)/$T60)/1000</f>
         <v/>
       </c>
+      <c r="AA60" s="47" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -32246,6 +32467,7 @@
         <f>((R61*8*1024)/$T61)/1000</f>
         <v/>
       </c>
+      <c r="AA61" s="48" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -32724,6 +32946,7 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
+      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -32810,6 +33033,7 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
+      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -32896,6 +33120,7 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
+      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -32982,6 +33207,7 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
+      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -33068,6 +33294,7 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
+      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -33154,6 +33381,7 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
+      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -33240,6 +33468,7 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
+      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -33335,6 +33564,7 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
+      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -33512,6 +33742,7 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
+      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -33598,6 +33829,7 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
+      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -33684,6 +33916,7 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
+      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -33770,6 +34003,7 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
+      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -33856,6 +34090,7 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
+      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -33938,6 +34173,7 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -34020,6 +34256,7 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -34102,6 +34339,7 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -34188,6 +34426,7 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
+      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -34274,6 +34513,7 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
+      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -34360,6 +34600,7 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
+      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -34446,6 +34687,7 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
+      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -34532,6 +34774,7 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
+      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -34618,6 +34861,7 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
+      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -34704,6 +34948,7 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
+      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -34790,6 +35035,7 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
+      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -34876,6 +35122,7 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
+      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -34962,6 +35209,7 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
+      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -35053,6 +35301,7 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
+      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -35139,6 +35388,7 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
+      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -35225,6 +35475,7 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
+      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -35311,6 +35562,7 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
+      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -35397,6 +35649,7 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
+      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -35483,6 +35736,7 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
+      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -35569,6 +35823,7 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
+      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -35655,6 +35910,7 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
+      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -35741,6 +35997,7 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
+      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -35836,6 +36093,7 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
+      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -36013,6 +36271,7 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
+      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -36099,6 +36358,7 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
+      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -36185,6 +36445,7 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
+      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -36271,6 +36532,7 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
+      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -36353,6 +36615,7 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
+      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -36439,6 +36702,7 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
+      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -36525,6 +36789,7 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
+      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -36611,6 +36876,7 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
+      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -36697,6 +36963,7 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
+      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -36783,6 +37050,7 @@
         <f>((R51*8*1024)/$T51)/1000</f>
         <v/>
       </c>
+      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -36869,6 +37137,7 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
+      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -36955,6 +37224,7 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
+      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -37041,6 +37311,7 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
+      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -37127,6 +37398,7 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
+      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -37213,6 +37485,7 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
+      <c r="AA56" s="47" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -37308,6 +37581,7 @@
         <f>100*(SUM(T47:T57))</f>
         <v/>
       </c>
+      <c r="AA57" s="47" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -37394,6 +37668,7 @@
         <f>((R58*8*1024)/$T58)/1000</f>
         <v/>
       </c>
+      <c r="AA58" s="47" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -37480,6 +37755,7 @@
         <f>((R59*8*1024)/$T59)/1000</f>
         <v/>
       </c>
+      <c r="AA59" s="48" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -37523,4 +37799,2442 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36.109375" customWidth="1" min="1" max="1"/>
+    <col width="20.44140625" customWidth="1" min="2" max="2"/>
+    <col width="4.109375" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="6.109375" customWidth="1" min="5" max="5"/>
+    <col width="11.6640625" customWidth="1" min="6" max="6"/>
+    <col width="5.44140625" customWidth="1" min="7" max="7"/>
+    <col width="6.109375" customWidth="1" min="8" max="8"/>
+    <col width="9.109375" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="5.44140625" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="6.109375" customWidth="1" min="14" max="14"/>
+    <col width="17.5546875" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="17.5546875" customWidth="1" min="17" max="17"/>
+    <col width="17.77734375" customWidth="1" min="18" max="18"/>
+    <col width="9.77734375" customWidth="1" min="19" max="19"/>
+    <col width="11.21875" customWidth="1" min="20" max="20"/>
+    <col width="10.88671875" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="10.5546875" customWidth="1" min="23" max="23"/>
+    <col width="12.77734375" customWidth="1" min="24" max="24"/>
+    <col width="30.33203125" customWidth="1" min="25" max="25"/>
+    <col width="12.77734375" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Cin</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Filter/Weight</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Cin</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Cout</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>BN</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="M1" s="14" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="N1" s="14" t="inlineStr">
+        <is>
+          <t>Cin</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Input 1 Memory(kB)</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Input 2 Memory(kB)</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>Input 3 Memory(kB)</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>Output Memory(kB)</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycles </t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>Time[us]</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>BW 1(Gbps)</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>BW 2(Gbps)</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>BW 3(Gbps)</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>BW Out(Gbps)</t>
+        </is>
+      </c>
+      <c r="Y1" s="19" t="inlineStr">
+        <is>
+          <t>freq Ghz</t>
+        </is>
+      </c>
+      <c r="Z1" s="16" t="inlineStr">
+        <is>
+          <t>Mem BW Gbps</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>kpt+desc load</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M2" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N2" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="3">
+        <f>C2*D2/1024</f>
+        <v/>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="3">
+        <f>L2*M2/1024</f>
+        <v/>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>KptEnc 3-&gt;32</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13" t="n">
+        <v>32</v>
+      </c>
+      <c r="M3" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3">
+        <f>C3*D3/1024</f>
+        <v/>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="3">
+        <f>L3*M3/1024</f>
+        <v/>
+      </c>
+      <c r="S3" s="3" t="n">
+        <v>3860</v>
+      </c>
+      <c r="T3" s="3">
+        <f>(S3/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U3" s="26">
+        <f>((O3*8*1024)/$T3)/1000</f>
+        <v/>
+      </c>
+      <c r="V3" s="26">
+        <f>((P3*8*1024)/$T3)/1000</f>
+        <v/>
+      </c>
+      <c r="W3" s="26">
+        <f>((Q3*8*1024)/$T3)/1000</f>
+        <v/>
+      </c>
+      <c r="X3" s="26">
+        <f>((R3*8*1024)/$T3)/1000</f>
+        <v/>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>KptEnc 32-&gt;64</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="13" t="n">
+        <v>64</v>
+      </c>
+      <c r="M4" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3">
+        <f>C4*D4/1024</f>
+        <v/>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="3">
+        <f>L4*M4/1024</f>
+        <v/>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>52265</v>
+      </c>
+      <c r="T4" s="3">
+        <f>(S4/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U4" s="26">
+        <f>((O4*8*1024)/$T4)/1000</f>
+        <v/>
+      </c>
+      <c r="V4" s="26">
+        <f>((P4*8*1024)/$T4)/1000</f>
+        <v/>
+      </c>
+      <c r="W4" s="26">
+        <f>((Q4*8*1024)/$T4)/1000</f>
+        <v/>
+      </c>
+      <c r="X4" s="26">
+        <f>((R4*8*1024)/$T4)/1000</f>
+        <v/>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>KptEnc 64-&gt;128</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="13" t="n">
+        <v>128</v>
+      </c>
+      <c r="M5" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="3">
+        <f>C5*D5/1024</f>
+        <v/>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="3">
+        <f>L5*M5/1024</f>
+        <v/>
+      </c>
+      <c r="S5" s="3" t="n">
+        <v>202834</v>
+      </c>
+      <c r="T5" s="3">
+        <f>(S5/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U5" s="26">
+        <f>((O5*8*1024)/$T5)/1000</f>
+        <v/>
+      </c>
+      <c r="V5" s="26">
+        <f>((P5*8*1024)/$T5)/1000</f>
+        <v/>
+      </c>
+      <c r="W5" s="26">
+        <f>((Q5*8*1024)/$T5)/1000</f>
+        <v/>
+      </c>
+      <c r="X5" s="26">
+        <f>((R5*8*1024)/$T5)/1000</f>
+        <v/>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>KptEnc 128-&gt;256</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>128</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M6" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="3">
+        <f>C6*D6/1024</f>
+        <v/>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="3">
+        <f>L6*M6/1024</f>
+        <v/>
+      </c>
+      <c r="S6" s="3" t="n">
+        <v>798884</v>
+      </c>
+      <c r="T6" s="3">
+        <f>(S6/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U6" s="26">
+        <f>((O6*8*1024)/$T6)/1000</f>
+        <v/>
+      </c>
+      <c r="V6" s="26">
+        <f>((P6*8*1024)/$T6)/1000</f>
+        <v/>
+      </c>
+      <c r="W6" s="26">
+        <f>((Q6*8*1024)/$T6)/1000</f>
+        <v/>
+      </c>
+      <c r="X6" s="26">
+        <f>((R6*8*1024)/$T6)/1000</f>
+        <v/>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Residual desc+=enc</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M7" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="3">
+        <f>C7*D7/1024</f>
+        <v/>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="3">
+        <f>L7*M7/1024</f>
+        <v/>
+      </c>
+      <c r="S7" s="3" t="n">
+        <v>10240</v>
+      </c>
+      <c r="T7" s="3">
+        <f>(S7/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U7" s="26">
+        <f>((O7*8*1024)/$T7)/1000</f>
+        <v/>
+      </c>
+      <c r="V7" s="26">
+        <f>((P7*8*1024)/$T7)/1000</f>
+        <v/>
+      </c>
+      <c r="W7" s="26">
+        <f>((Q7*8*1024)/$T7)/1000</f>
+        <v/>
+      </c>
+      <c r="X7" s="26">
+        <f>((R7*8*1024)/$T7)/1000</f>
+        <v/>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Q proj D-&gt;D</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M8" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="3">
+        <f>C8*D8/1024</f>
+        <v/>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="3">
+        <f>L8*M8/1024</f>
+        <v/>
+      </c>
+      <c r="S8" s="3" t="n">
+        <v>28535685</v>
+      </c>
+      <c r="T8" s="3">
+        <f>(S8/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U8" s="26">
+        <f>((O8*8*1024)/$T8)/1000</f>
+        <v/>
+      </c>
+      <c r="V8" s="26">
+        <f>((P8*8*1024)/$T8)/1000</f>
+        <v/>
+      </c>
+      <c r="W8" s="26">
+        <f>((Q8*8*1024)/$T8)/1000</f>
+        <v/>
+      </c>
+      <c r="X8" s="26">
+        <f>((R8*8*1024)/$T8)/1000</f>
+        <v/>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>K proj D-&gt;D</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="3">
+        <f>C9*D9/1024</f>
+        <v/>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="3">
+        <f>L9*M9/1024</f>
+        <v/>
+      </c>
+      <c r="S9" s="3" t="n">
+        <v>28535685</v>
+      </c>
+      <c r="T9" s="3">
+        <f>(S9/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U9" s="26">
+        <f>((O9*8*1024)/$T9)/1000</f>
+        <v/>
+      </c>
+      <c r="V9" s="26">
+        <f>((P9*8*1024)/$T9)/1000</f>
+        <v/>
+      </c>
+      <c r="W9" s="26">
+        <f>((Q9*8*1024)/$T9)/1000</f>
+        <v/>
+      </c>
+      <c r="X9" s="26">
+        <f>((R9*8*1024)/$T9)/1000</f>
+        <v/>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>V proj D-&gt;D</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M10" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="3">
+        <f>C10*D10/1024</f>
+        <v/>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="3">
+        <f>L10*M10/1024</f>
+        <v/>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>28535685</v>
+      </c>
+      <c r="T10" s="3">
+        <f>(S10/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U10" s="26">
+        <f>((O10*8*1024)/$T10)/1000</f>
+        <v/>
+      </c>
+      <c r="V10" s="26">
+        <f>((P10*8*1024)/$T10)/1000</f>
+        <v/>
+      </c>
+      <c r="W10" s="26">
+        <f>((Q10*8*1024)/$T10)/1000</f>
+        <v/>
+      </c>
+      <c r="X10" s="26">
+        <f>((R10*8*1024)/$T10)/1000</f>
+        <v/>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>QKt</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="3">
+        <f>C11*D11/1024</f>
+        <v/>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="3">
+        <f>L11*M11/1024</f>
+        <v/>
+      </c>
+      <c r="S11" s="3" t="n">
+        <v>58416169</v>
+      </c>
+      <c r="T11" s="3">
+        <f>(S11/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U11" s="26">
+        <f>((O11*8*1024)/$T11)/1000</f>
+        <v/>
+      </c>
+      <c r="V11" s="26">
+        <f>((P11*8*1024)/$T11)/1000</f>
+        <v/>
+      </c>
+      <c r="W11" s="26">
+        <f>((Q11*8*1024)/$T11)/1000</f>
+        <v/>
+      </c>
+      <c r="X11" s="26">
+        <f>((R11*8*1024)/$T11)/1000</f>
+        <v/>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>x144</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>scale 1/sqrt(d)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>multiply</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="M12" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="3">
+        <f>C12*D12/1024</f>
+        <v/>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="3">
+        <f>L12*M12/1024</f>
+        <v/>
+      </c>
+      <c r="S12" s="3" t="n">
+        <v>1474560</v>
+      </c>
+      <c r="T12" s="3">
+        <f>(S12/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U12" s="26">
+        <f>((O12*8*1024)/$T12)/1000</f>
+        <v/>
+      </c>
+      <c r="V12" s="26">
+        <f>((P12*8*1024)/$T12)/1000</f>
+        <v/>
+      </c>
+      <c r="W12" s="26">
+        <f>((Q12*8*1024)/$T12)/1000</f>
+        <v/>
+      </c>
+      <c r="X12" s="26">
+        <f>((R12*8*1024)/$T12)/1000</f>
+        <v/>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>x144</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>softmax</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>max,exp2,sum,mul</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="3">
+        <f>C13*D13/1024</f>
+        <v/>
+      </c>
+      <c r="P13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="3">
+        <f>L13*M13/1024</f>
+        <v/>
+      </c>
+      <c r="S13" s="3" t="n">
+        <v>5603328</v>
+      </c>
+      <c r="T13" s="3">
+        <f>(S13/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U13" s="26">
+        <f>((O13*8*1024)/$T13)/1000</f>
+        <v/>
+      </c>
+      <c r="V13" s="26">
+        <f>((P13*8*1024)/$T13)/1000</f>
+        <v/>
+      </c>
+      <c r="W13" s="26">
+        <f>((Q13*8*1024)/$T13)/1000</f>
+        <v/>
+      </c>
+      <c r="X13" s="26">
+        <f>((R13*8*1024)/$T13)/1000</f>
+        <v/>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>x144</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>attn @ V</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>512</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>64</v>
+      </c>
+      <c r="N14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="3">
+        <f>C14*D14/1024</f>
+        <v/>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="3">
+        <f>L14*M14/1024</f>
+        <v/>
+      </c>
+      <c r="S14" s="3" t="n">
+        <v>56847237</v>
+      </c>
+      <c r="T14" s="3">
+        <f>(S14/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U14" s="26">
+        <f>((O14*8*1024)/$T14)/1000</f>
+        <v/>
+      </c>
+      <c r="V14" s="26">
+        <f>((P14*8*1024)/$T14)/1000</f>
+        <v/>
+      </c>
+      <c r="W14" s="26">
+        <f>((Q14*8*1024)/$T14)/1000</f>
+        <v/>
+      </c>
+      <c r="X14" s="26">
+        <f>((R14*8*1024)/$T14)/1000</f>
+        <v/>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>x144</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>out proj D-&gt;D</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="3">
+        <f>C15*D15/1024</f>
+        <v/>
+      </c>
+      <c r="P15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="3">
+        <f>L15*M15/1024</f>
+        <v/>
+      </c>
+      <c r="S15" s="3" t="n">
+        <v>28535685</v>
+      </c>
+      <c r="T15" s="3">
+        <f>(S15/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U15" s="26">
+        <f>((O15*8*1024)/$T15)/1000</f>
+        <v/>
+      </c>
+      <c r="V15" s="26">
+        <f>((P15*8*1024)/$T15)/1000</f>
+        <v/>
+      </c>
+      <c r="W15" s="26">
+        <f>((Q15*8*1024)/$T15)/1000</f>
+        <v/>
+      </c>
+      <c r="X15" s="26">
+        <f>((R15*8*1024)/$T15)/1000</f>
+        <v/>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Residual x+=msg</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="3">
+        <f>C16*D16/1024</f>
+        <v/>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="3">
+        <f>L16*M16/1024</f>
+        <v/>
+      </c>
+      <c r="S16" s="3" t="n">
+        <v>184320</v>
+      </c>
+      <c r="T16" s="3">
+        <f>(S16/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U16" s="26">
+        <f>((O16*8*1024)/$T16)/1000</f>
+        <v/>
+      </c>
+      <c r="V16" s="26">
+        <f>((P16*8*1024)/$T16)/1000</f>
+        <v/>
+      </c>
+      <c r="W16" s="26">
+        <f>((Q16*8*1024)/$T16)/1000</f>
+        <v/>
+      </c>
+      <c r="X16" s="26">
+        <f>((R16*8*1024)/$T16)/1000</f>
+        <v/>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>merge MLP 2D-&gt;2D</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>512</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="M17" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N17" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="3">
+        <f>C17*D17/1024</f>
+        <v/>
+      </c>
+      <c r="P17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="3">
+        <f>L17*M17/1024</f>
+        <v/>
+      </c>
+      <c r="S17" s="3" t="n">
+        <v>113694474</v>
+      </c>
+      <c r="T17" s="3">
+        <f>(S17/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U17" s="26">
+        <f>((O17*8*1024)/$T17)/1000</f>
+        <v/>
+      </c>
+      <c r="V17" s="26">
+        <f>((P17*8*1024)/$T17)/1000</f>
+        <v/>
+      </c>
+      <c r="W17" s="26">
+        <f>((Q17*8*1024)/$T17)/1000</f>
+        <v/>
+      </c>
+      <c r="X17" s="26">
+        <f>((R17*8*1024)/$T17)/1000</f>
+        <v/>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>merge MLP relu</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="M18" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N18" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="3">
+        <f>C18*D18/1024</f>
+        <v/>
+      </c>
+      <c r="P18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="3">
+        <f>L18*M18/1024</f>
+        <v/>
+      </c>
+      <c r="S18" s="3" t="n">
+        <v>368640</v>
+      </c>
+      <c r="T18" s="3">
+        <f>(S18/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U18" s="26">
+        <f>((O18*8*1024)/$T18)/1000</f>
+        <v/>
+      </c>
+      <c r="V18" s="26">
+        <f>((P18*8*1024)/$T18)/1000</f>
+        <v/>
+      </c>
+      <c r="W18" s="26">
+        <f>((Q18*8*1024)/$T18)/1000</f>
+        <v/>
+      </c>
+      <c r="X18" s="26">
+        <f>((R18*8*1024)/$T18)/1000</f>
+        <v/>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>merge MLP 2D-&gt;D</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>512</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M19" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="3">
+        <f>C19*D19/1024</f>
+        <v/>
+      </c>
+      <c r="P19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="3">
+        <f>L19*M19/1024</f>
+        <v/>
+      </c>
+      <c r="S19" s="3" t="n">
+        <v>56847237</v>
+      </c>
+      <c r="T19" s="3">
+        <f>(S19/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U19" s="26">
+        <f>((O19*8*1024)/$T19)/1000</f>
+        <v/>
+      </c>
+      <c r="V19" s="26">
+        <f>((P19*8*1024)/$T19)/1000</f>
+        <v/>
+      </c>
+      <c r="W19" s="26">
+        <f>((Q19*8*1024)/$T19)/1000</f>
+        <v/>
+      </c>
+      <c r="X19" s="26">
+        <f>((R19*8*1024)/$T19)/1000</f>
+        <v/>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Residual x+=mlp</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="3">
+        <f>C20*D20/1024</f>
+        <v/>
+      </c>
+      <c r="P20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="3">
+        <f>L20*M20/1024</f>
+        <v/>
+      </c>
+      <c r="S20" s="3" t="n">
+        <v>184320</v>
+      </c>
+      <c r="T20" s="3">
+        <f>(S20/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U20" s="26">
+        <f>((O20*8*1024)/$T20)/1000</f>
+        <v/>
+      </c>
+      <c r="V20" s="26">
+        <f>((P20*8*1024)/$T20)/1000</f>
+        <v/>
+      </c>
+      <c r="W20" s="26">
+        <f>((Q20*8*1024)/$T20)/1000</f>
+        <v/>
+      </c>
+      <c r="X20" s="26">
+        <f>((R20*8*1024)/$T20)/1000</f>
+        <v/>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>x36</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>final proj D-&gt;D</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="13" t="n">
+        <v>256</v>
+      </c>
+      <c r="M21" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="3">
+        <f>C21*D21/1024</f>
+        <v/>
+      </c>
+      <c r="P21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="3">
+        <f>L21*M21/1024</f>
+        <v/>
+      </c>
+      <c r="S21" s="3" t="n">
+        <v>1585316</v>
+      </c>
+      <c r="T21" s="3">
+        <f>(S21/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U21" s="26">
+        <f>((O21*8*1024)/$T21)/1000</f>
+        <v/>
+      </c>
+      <c r="V21" s="26">
+        <f>((P21*8*1024)/$T21)/1000</f>
+        <v/>
+      </c>
+      <c r="W21" s="26">
+        <f>((Q21*8*1024)/$T21)/1000</f>
+        <v/>
+      </c>
+      <c r="X21" s="26">
+        <f>((R21*8*1024)/$T21)/1000</f>
+        <v/>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>score = A^T B</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>MAC matmul</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>256</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="M22" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N22" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="3">
+        <f>C22*D22/1024</f>
+        <v/>
+      </c>
+      <c r="P22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="3">
+        <f>L22*M22/1024</f>
+        <v/>
+      </c>
+      <c r="S22" s="3" t="n">
+        <v>1585316</v>
+      </c>
+      <c r="T22" s="3">
+        <f>(S22/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U22" s="26">
+        <f>((O22*8*1024)/$T22)/1000</f>
+        <v/>
+      </c>
+      <c r="V22" s="26">
+        <f>((P22*8*1024)/$T22)/1000</f>
+        <v/>
+      </c>
+      <c r="W22" s="26">
+        <f>((Q22*8*1024)/$T22)/1000</f>
+        <v/>
+      </c>
+      <c r="X22" s="26">
+        <f>((R22*8*1024)/$T22)/1000</f>
+        <v/>
+      </c>
+      <c r="Y22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>scale 1/sqrt(d)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>multiply</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>512</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="M23" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="N23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="3">
+        <f>C23*D23/1024</f>
+        <v/>
+      </c>
+      <c r="P23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="3">
+        <f>L23*M23/1024</f>
+        <v/>
+      </c>
+      <c r="S23" s="3" t="n">
+        <v>10240</v>
+      </c>
+      <c r="T23" s="3">
+        <f>(S23/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U23" s="26">
+        <f>((O23*8*1024)/$T23)/1000</f>
+        <v/>
+      </c>
+      <c r="V23" s="26">
+        <f>((P23*8*1024)/$T23)/1000</f>
+        <v/>
+      </c>
+      <c r="W23" s="26">
+        <f>((Q23*8*1024)/$T23)/1000</f>
+        <v/>
+      </c>
+      <c r="X23" s="26">
+        <f>((R23*8*1024)/$T23)/1000</f>
+        <v/>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Sinkhorn row norm (max)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>sum,scale</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>513</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>513</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="13" t="n">
+        <v>513</v>
+      </c>
+      <c r="M24" s="13" t="n">
+        <v>513</v>
+      </c>
+      <c r="N24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="3">
+        <f>C24*D24/1024</f>
+        <v/>
+      </c>
+      <c r="P24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="3">
+        <f>L24*M24/1024</f>
+        <v/>
+      </c>
+      <c r="S24" s="3" t="n">
+        <v>2336555</v>
+      </c>
+      <c r="T24" s="3">
+        <f>(S24/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U24" s="26">
+        <f>((O24*8*1024)/$T24)/1000</f>
+        <v/>
+      </c>
+      <c r="V24" s="26">
+        <f>((P24*8*1024)/$T24)/1000</f>
+        <v/>
+      </c>
+      <c r="W24" s="26">
+        <f>((Q24*8*1024)/$T24)/1000</f>
+        <v/>
+      </c>
+      <c r="X24" s="26">
+        <f>((R24*8*1024)/$T24)/1000</f>
+        <v/>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>x100</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Sinkhorn col norm (max)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>ACC.MAX,scale</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>513</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <v>513</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="13" t="n">
+        <v>513</v>
+      </c>
+      <c r="M25" s="13" t="n">
+        <v>513</v>
+      </c>
+      <c r="N25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="3">
+        <f>C25*D25/1024</f>
+        <v/>
+      </c>
+      <c r="P25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="3">
+        <f>L25*M25/1024</f>
+        <v/>
+      </c>
+      <c r="S25" s="3" t="n">
+        <v>4176141</v>
+      </c>
+      <c r="T25" s="3">
+        <f>(S25/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U25" s="26">
+        <f>((O25*8*1024)/$T25)/1000</f>
+        <v/>
+      </c>
+      <c r="V25" s="26">
+        <f>((P25*8*1024)/$T25)/1000</f>
+        <v/>
+      </c>
+      <c r="W25" s="26">
+        <f>((Q25*8*1024)/$T25)/1000</f>
+        <v/>
+      </c>
+      <c r="X25" s="26">
+        <f>((R25*8*1024)/$T25)/1000</f>
+        <v/>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>x100</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>match readout</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>argmax+thresh</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>513</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>513</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="13" t="n">
+        <v>513</v>
+      </c>
+      <c r="M26" s="13" t="n">
+        <v>513</v>
+      </c>
+      <c r="N26" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="3">
+        <f>C26*D26/1024</f>
+        <v/>
+      </c>
+      <c r="P26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="3">
+        <f>L26*M26/1024</f>
+        <v/>
+      </c>
+      <c r="S26" s="3" t="n">
+        <v>10285</v>
+      </c>
+      <c r="T26" s="3">
+        <f>(S26/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U26" s="26">
+        <f>((O26*8*1024)/$T26)/1000</f>
+        <v/>
+      </c>
+      <c r="V26" s="26">
+        <f>((P26*8*1024)/$T26)/1000</f>
+        <v/>
+      </c>
+      <c r="W26" s="26">
+        <f>((Q26*8*1024)/$T26)/1000</f>
+        <v/>
+      </c>
+      <c r="X26" s="26">
+        <f>((R26*8*1024)/$T26)/1000</f>
+        <v/>
+      </c>
+      <c r="Y26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL [us] (measured)</t>
+        </is>
+      </c>
+      <c r="Y27" s="17" t="inlineStr">
+        <is>
+          <t>measured emulator cycles -&gt;</t>
+        </is>
+      </c>
+      <c r="Z27" s="17">
+        <f>SUM(T2:T26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>FPS (image pair)</t>
+        </is>
+      </c>
+      <c r="Y28" s="17" t="inlineStr">
+        <is>
+          <t>frames / sec -&gt;</t>
+        </is>
+      </c>
+      <c r="Z28" s="17">
+        <f>1000000/Z27</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
build_sg_excel.py: single from-scratch SuperGlue Excel builder + self-validation
Replaces build_superglue_xlsx.py and add_measured_sheet.py (deleted) with one
clean script that builds the whole workbook from scratch off a MobileViT
template and SELF-VALIDATES every sheet: an independent Python re-computation
of each variant's grand-total cycles is cross-checked against the spreadsheet's
formula-evaluated Z cell. All six sheets PASS (PY model == XLS formula at FP
precision):
  SuperGlue (original)            271220.9 us   3.69 FPS
  SG max-Sinkhorn                 269987.3 us   3.70 FPS
  SG base2-softmax                271220.9 us   3.69 FPS
  SG transpose-free col           271015.3 us   3.69 FPS
  SG fixed-thresh match           271214.7 us   3.69 FPS
  SG max-Sinkhorn (measured)      418535.0 us   2.39 FPS  (emulator rates)

Source is the uploaded cb06a587-IPU_2.xlsx (MobileViT-only template); output is
IPU_2_SuperGlue.xlsx.

https://claude.ai/code/session_01Wj1AhpfDtCg3YHVUGoUUbF
</commit_message>
<xml_diff>
--- a/IPU_2_SuperGlue.xlsx
+++ b/IPU_2_SuperGlue.xlsx
@@ -10932,7 +10932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA65"/>
+  <dimension ref="A1:Z65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36.109375" customWidth="1" min="1" max="1"/>
@@ -11268,11 +11268,6 @@
         <f>((R3*8*1024)/$T3)/1000</f>
         <v/>
       </c>
-      <c r="AA3" s="44" t="inlineStr">
-        <is>
-          <t>Keypoint Encoder (x2 images)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -11359,7 +11354,6 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
-      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -11446,7 +11440,6 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
-      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -11533,7 +11526,6 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
-      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -11620,7 +11612,6 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
-      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -11707,7 +11698,6 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
-      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -11794,7 +11784,6 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
-      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -11881,7 +11870,6 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
-      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -11977,7 +11965,6 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
-      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -12064,11 +12051,6 @@
         <f>((R12*8*1024)/$T12)/1000</f>
         <v/>
       </c>
-      <c r="AA12" s="44" t="inlineStr">
-        <is>
-          <t>Attentional GNN block (x36=18 layers x2 img)</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -12155,7 +12137,6 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
-      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -12242,7 +12223,6 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
-      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -12329,7 +12309,6 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
-      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -12416,7 +12395,6 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
-      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -12503,7 +12481,6 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
-      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -12586,7 +12563,6 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -12669,7 +12645,6 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -12752,7 +12727,6 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -12839,7 +12813,6 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
-      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -12926,7 +12899,6 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
-      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -13013,7 +12985,6 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
-      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -13100,7 +13071,6 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
-      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -13187,7 +13157,6 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
-      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -13274,7 +13243,6 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
-      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -13361,7 +13329,6 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
-      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -13448,7 +13415,6 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
-      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -13535,7 +13501,6 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
-      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -13622,7 +13587,6 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
-      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -13714,7 +13678,6 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
-      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -13801,7 +13764,6 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
-      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -13888,7 +13850,6 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
-      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -13975,7 +13936,6 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
-      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -14062,7 +14022,6 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
-      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -14149,7 +14108,6 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
-      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -14236,7 +14194,6 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
-      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -14323,7 +14280,6 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
-      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -14410,7 +14366,6 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
-      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -14506,7 +14461,6 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
-      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -14593,11 +14547,6 @@
         <f>((R41*8*1024)/$T41)/1000</f>
         <v/>
       </c>
-      <c r="AA41" s="44" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -14684,7 +14633,6 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
-      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -14771,7 +14719,6 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
-      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -14858,7 +14805,6 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
-      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -14945,7 +14891,6 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
-      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -15028,7 +14973,6 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -15115,7 +15059,6 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
-      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -15202,7 +15145,6 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
-      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -15289,7 +15231,6 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
-      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -15376,7 +15317,6 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
-      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -15463,7 +15403,6 @@
         <f>((R51*8*1024)/$T51)/1000</f>
         <v/>
       </c>
-      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -15550,7 +15489,6 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
-      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -15637,7 +15575,6 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
-      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -15724,7 +15661,6 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
-      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -15811,7 +15747,6 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
-      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -15898,7 +15833,6 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
-      <c r="AA56" s="47" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -15994,7 +15928,6 @@
         <f>100*(SUM(T47:T57))</f>
         <v/>
       </c>
-      <c r="AA57" s="47" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -16081,7 +16014,6 @@
         <f>((R58*8*1024)/$T58)/1000</f>
         <v/>
       </c>
-      <c r="AA58" s="47" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -16168,7 +16100,6 @@
         <f>((R59*8*1024)/$T59)/1000</f>
         <v/>
       </c>
-      <c r="AA59" s="47" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -16255,7 +16186,6 @@
         <f>((R60*8*1024)/$T60)/1000</f>
         <v/>
       </c>
-      <c r="AA60" s="47" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -16342,7 +16272,6 @@
         <f>((R61*8*1024)/$T61)/1000</f>
         <v/>
       </c>
-      <c r="AA61" s="47" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -16429,7 +16358,6 @@
         <f>((R62*8*1024)/$T62)/1000</f>
         <v/>
       </c>
-      <c r="AA62" s="48" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -16464,13 +16392,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="AA47:AA57"/>
-    <mergeCell ref="AA21:AA30"/>
-    <mergeCell ref="AA12:AA40"/>
-    <mergeCell ref="AA3:AA11"/>
-    <mergeCell ref="AA41:AA62"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16481,7 +16402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA59"/>
+  <dimension ref="A1:Z59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36.109375" customWidth="1" min="1" max="1"/>
@@ -16817,11 +16738,6 @@
         <f>((R3*8*1024)/$T3)/1000</f>
         <v/>
       </c>
-      <c r="AA3" s="44" t="inlineStr">
-        <is>
-          <t>Keypoint Encoder (x2 images)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -16908,7 +16824,6 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
-      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -16995,7 +16910,6 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
-      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -17082,7 +16996,6 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
-      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -17169,7 +17082,6 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
-      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -17256,7 +17168,6 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
-      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -17343,7 +17254,6 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
-      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -17430,7 +17340,6 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
-      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -17526,7 +17435,6 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
-      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -17613,11 +17521,6 @@
         <f>((R12*8*1024)/$T12)/1000</f>
         <v/>
       </c>
-      <c r="AA12" s="44" t="inlineStr">
-        <is>
-          <t>Attentional GNN block (x36=18 layers x2 img)</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -17704,7 +17607,6 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
-      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -17791,7 +17693,6 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
-      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -17878,7 +17779,6 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
-      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -17965,7 +17865,6 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
-      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -18052,7 +17951,6 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
-      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -18135,7 +18033,6 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -18218,7 +18115,6 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -18301,7 +18197,6 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -18388,7 +18283,6 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
-      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -18475,7 +18369,6 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
-      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -18562,7 +18455,6 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
-      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -18649,7 +18541,6 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
-      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -18736,7 +18627,6 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
-      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -18823,7 +18713,6 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
-      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -18910,7 +18799,6 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
-      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -18997,7 +18885,6 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
-      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -19084,7 +18971,6 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
-      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -19171,7 +19057,6 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
-      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -19263,7 +19148,6 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
-      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -19350,7 +19234,6 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
-      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -19437,7 +19320,6 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
-      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -19524,7 +19406,6 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
-      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -19611,7 +19492,6 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
-      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -19698,7 +19578,6 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
-      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -19785,7 +19664,6 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
-      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -19872,7 +19750,6 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
-      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -19959,7 +19836,6 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
-      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -20055,7 +19931,6 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
-      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -20142,11 +20017,6 @@
         <f>((R41*8*1024)/$T41)/1000</f>
         <v/>
       </c>
-      <c r="AA41" s="44" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -20233,7 +20103,6 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
-      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -20320,7 +20189,6 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
-      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -20407,7 +20275,6 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
-      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -20494,7 +20361,6 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
-      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -20577,7 +20443,6 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -20664,7 +20529,6 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
-      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -20751,7 +20615,6 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
-      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -20838,7 +20701,6 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
-      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -20925,7 +20787,6 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
-      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -21021,7 +20882,6 @@
         <f>100*(SUM(T47:T51))</f>
         <v/>
       </c>
-      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -21108,7 +20968,6 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
-      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -21195,7 +21054,6 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
-      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -21282,7 +21140,6 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
-      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -21369,7 +21226,6 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
-      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -21456,7 +21312,6 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
-      <c r="AA56" s="48" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -21491,13 +21346,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="AA21:AA30"/>
-    <mergeCell ref="AA12:AA40"/>
-    <mergeCell ref="AA3:AA11"/>
-    <mergeCell ref="AA41:AA56"/>
-    <mergeCell ref="AA47:AA51"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21508,7 +21356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA65"/>
+  <dimension ref="A1:Z65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36.109375" customWidth="1" min="1" max="1"/>
@@ -21844,11 +21692,6 @@
         <f>((R3*8*1024)/$T3)/1000</f>
         <v/>
       </c>
-      <c r="AA3" s="44" t="inlineStr">
-        <is>
-          <t>Keypoint Encoder (x2 images)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -21935,7 +21778,6 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
-      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -22022,7 +21864,6 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
-      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -22109,7 +21950,6 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
-      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -22196,7 +22036,6 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
-      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -22283,7 +22122,6 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
-      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -22370,7 +22208,6 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
-      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -22457,7 +22294,6 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
-      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -22553,7 +22389,6 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
-      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -22640,11 +22475,6 @@
         <f>((R12*8*1024)/$T12)/1000</f>
         <v/>
       </c>
-      <c r="AA12" s="44" t="inlineStr">
-        <is>
-          <t>Attentional GNN block (x36=18 layers x2 img)</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -22731,7 +22561,6 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
-      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -22818,7 +22647,6 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
-      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -22905,7 +22733,6 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
-      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -22992,7 +22819,6 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
-      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -23079,7 +22905,6 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
-      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -23162,7 +22987,6 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -23245,7 +23069,6 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -23328,7 +23151,6 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -23415,7 +23237,6 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
-      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -23502,7 +23323,6 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
-      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -23589,7 +23409,6 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
-      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -23676,7 +23495,6 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
-      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -23763,7 +23581,6 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
-      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -23850,7 +23667,6 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
-      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -23937,7 +23753,6 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
-      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -24024,7 +23839,6 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
-      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -24111,7 +23925,6 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
-      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -24198,7 +24011,6 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
-      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -24290,7 +24102,6 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
-      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -24377,7 +24188,6 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
-      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -24464,7 +24274,6 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
-      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -24551,7 +24360,6 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
-      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -24638,7 +24446,6 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
-      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -24725,7 +24532,6 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
-      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -24812,7 +24618,6 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
-      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -24899,7 +24704,6 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
-      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -24986,7 +24790,6 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
-      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -25082,7 +24885,6 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
-      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -25169,11 +24971,6 @@
         <f>((R41*8*1024)/$T41)/1000</f>
         <v/>
       </c>
-      <c r="AA41" s="44" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -25260,7 +25057,6 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
-      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -25347,7 +25143,6 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
-      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -25434,7 +25229,6 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
-      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -25521,7 +25315,6 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
-      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -25604,7 +25397,6 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -25691,7 +25483,6 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
-      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -25778,7 +25569,6 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
-      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -25865,7 +25655,6 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
-      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -25952,7 +25741,6 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
-      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -26039,7 +25827,6 @@
         <f>((R51*8*1024)/$T51)/1000</f>
         <v/>
       </c>
-      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -26126,7 +25913,6 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
-      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -26213,7 +25999,6 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
-      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -26300,7 +26085,6 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
-      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -26387,7 +26171,6 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
-      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -26474,7 +26257,6 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
-      <c r="AA56" s="47" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -26570,7 +26352,6 @@
         <f>100*(SUM(T47:T57))</f>
         <v/>
       </c>
-      <c r="AA57" s="47" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -26657,7 +26438,6 @@
         <f>((R58*8*1024)/$T58)/1000</f>
         <v/>
       </c>
-      <c r="AA58" s="47" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -26744,7 +26524,6 @@
         <f>((R59*8*1024)/$T59)/1000</f>
         <v/>
       </c>
-      <c r="AA59" s="47" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -26831,7 +26610,6 @@
         <f>((R60*8*1024)/$T60)/1000</f>
         <v/>
       </c>
-      <c r="AA60" s="47" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -26918,7 +26696,6 @@
         <f>((R61*8*1024)/$T61)/1000</f>
         <v/>
       </c>
-      <c r="AA61" s="47" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -27005,7 +26782,6 @@
         <f>((R62*8*1024)/$T62)/1000</f>
         <v/>
       </c>
-      <c r="AA62" s="48" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -27040,13 +26816,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="AA47:AA57"/>
-    <mergeCell ref="AA21:AA30"/>
-    <mergeCell ref="AA12:AA40"/>
-    <mergeCell ref="AA3:AA11"/>
-    <mergeCell ref="AA41:AA62"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27057,7 +26826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA64"/>
+  <dimension ref="A1:Z65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36.109375" customWidth="1" min="1" max="1"/>
@@ -27393,11 +27162,6 @@
         <f>((R3*8*1024)/$T3)/1000</f>
         <v/>
       </c>
-      <c r="AA3" s="44" t="inlineStr">
-        <is>
-          <t>Keypoint Encoder (x2 images)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -27484,7 +27248,6 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
-      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -27571,7 +27334,6 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
-      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -27658,7 +27420,6 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
-      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -27745,7 +27506,6 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
-      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -27832,7 +27592,6 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
-      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -27919,7 +27678,6 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
-      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -28006,7 +27764,6 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
-      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -28102,7 +27859,6 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
-      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -28189,11 +27945,6 @@
         <f>((R12*8*1024)/$T12)/1000</f>
         <v/>
       </c>
-      <c r="AA12" s="44" t="inlineStr">
-        <is>
-          <t>Attentional GNN block (x36=18 layers x2 img)</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -28280,7 +28031,6 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
-      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -28367,7 +28117,6 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
-      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -28454,7 +28203,6 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
-      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -28541,7 +28289,6 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
-      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -28628,7 +28375,6 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
-      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -28711,7 +28457,6 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -28794,7 +28539,6 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -28877,7 +28621,6 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -28964,7 +28707,6 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
-      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -29051,7 +28793,6 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
-      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -29138,7 +28879,6 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
-      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -29225,7 +28965,6 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
-      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -29312,7 +29051,6 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
-      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -29399,7 +29137,6 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
-      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -29486,7 +29223,6 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
-      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -29573,7 +29309,6 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
-      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -29660,7 +29395,6 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
-      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -29747,7 +29481,6 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
-      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -29839,7 +29572,6 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
-      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -29926,7 +29658,6 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
-      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -30013,7 +29744,6 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
-      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -30100,7 +29830,6 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
-      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -30187,7 +29916,6 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
-      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -30274,7 +30002,6 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
-      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -30361,7 +30088,6 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
-      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -30448,7 +30174,6 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
-      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -30535,7 +30260,6 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
-      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -30631,7 +30355,6 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
-      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -30718,11 +30441,6 @@
         <f>((R41*8*1024)/$T41)/1000</f>
         <v/>
       </c>
-      <c r="AA41" s="44" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -30809,7 +30527,6 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
-      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -30896,7 +30613,6 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
-      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -30983,7 +30699,6 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
-      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -31070,7 +30785,6 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
-      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -31153,7 +30867,6 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -31240,7 +30953,6 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
-      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -31327,7 +31039,6 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
-      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -31414,7 +31125,6 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
-      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -31501,7 +31211,6 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
-      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -31588,17 +31297,16 @@
         <f>((R51*8*1024)/$T51)/1000</f>
         <v/>
       </c>
-      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>Sinkhorn col norm</t>
+          <t>Sinkhorn col transpose (eliminated)</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>reshape</t>
         </is>
       </c>
       <c r="C52" s="11" t="n">
@@ -31651,31 +31359,26 @@
         <f>L52*M52/1024</f>
         <v/>
       </c>
-      <c r="S52" s="3">
-        <f>C52*D52/128</f>
-        <v/>
-      </c>
-      <c r="T52" s="3">
-        <f>(S52/$Y$2)/1000</f>
-        <v/>
-      </c>
-      <c r="U52" s="26">
-        <f>((O52*8*1024)/$T52)/1000</f>
-        <v/>
-      </c>
-      <c r="V52" s="26">
-        <f>((P52*8*1024)/$T52)/1000</f>
-        <v/>
-      </c>
-      <c r="W52" s="26">
-        <f>((Q52*8*1024)/$T52)/1000</f>
-        <v/>
-      </c>
-      <c r="X52" s="26">
-        <f>((R52*8*1024)/$T52)/1000</f>
-        <v/>
-      </c>
-      <c r="AA52" s="47" t="n"/>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U52" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="V52" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="W52" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X52" s="26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -31685,7 +31388,7 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>exp2</t>
+          <t>max</t>
         </is>
       </c>
       <c r="C53" s="11" t="n">
@@ -31762,7 +31465,6 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
-      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -31772,7 +31474,7 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>sum</t>
+          <t>exp2</t>
         </is>
       </c>
       <c r="C54" s="11" t="n">
@@ -31849,7 +31551,6 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
-      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -31859,7 +31560,7 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>log</t>
+          <t>sum</t>
         </is>
       </c>
       <c r="C55" s="11" t="n">
@@ -31936,7 +31637,6 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
-      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -31946,7 +31646,7 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>subtract</t>
+          <t>log</t>
         </is>
       </c>
       <c r="C56" s="11" t="n">
@@ -32023,26 +31723,16 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
-      <c r="Y56" s="17" t="inlineStr">
-        <is>
-          <t>Sinkhorn total (x100) [us] -&gt;</t>
-        </is>
-      </c>
-      <c r="Z56" s="17">
-        <f>100*(SUM(T47:T56))</f>
-        <v/>
-      </c>
-      <c r="AA56" s="47" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>match readout (dual-softmax)</t>
+          <t>Sinkhorn col norm</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>subtract</t>
         </is>
       </c>
       <c r="C57" s="11" t="n">
@@ -32119,7 +31809,15 @@
         <f>((R57*8*1024)/$T57)/1000</f>
         <v/>
       </c>
-      <c r="AA57" s="47" t="n"/>
+      <c r="Y57" s="17" t="inlineStr">
+        <is>
+          <t>Sinkhorn total (x100) [us] -&gt;</t>
+        </is>
+      </c>
+      <c r="Z57" s="17">
+        <f>100*(SUM(T47:T57))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -32129,7 +31827,7 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>exp2</t>
+          <t>max</t>
         </is>
       </c>
       <c r="C58" s="11" t="n">
@@ -32206,7 +31904,6 @@
         <f>((R58*8*1024)/$T58)/1000</f>
         <v/>
       </c>
-      <c r="AA58" s="47" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -32216,7 +31913,7 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>sum</t>
+          <t>exp2</t>
         </is>
       </c>
       <c r="C59" s="11" t="n">
@@ -32293,7 +31990,6 @@
         <f>((R59*8*1024)/$T59)/1000</f>
         <v/>
       </c>
-      <c r="AA59" s="47" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -32303,7 +31999,7 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>subtract</t>
+          <t>sum</t>
         </is>
       </c>
       <c r="C60" s="11" t="n">
@@ -32380,7 +32076,6 @@
         <f>((R60*8*1024)/$T60)/1000</f>
         <v/>
       </c>
-      <c r="AA60" s="47" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -32390,7 +32085,7 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>multiply</t>
+          <t>subtract</t>
         </is>
       </c>
       <c r="C61" s="11" t="n">
@@ -32467,48 +32162,126 @@
         <f>((R61*8*1024)/$T61)/1000</f>
         <v/>
       </c>
-      <c r="AA61" s="48" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL [us]</t>
-        </is>
-      </c>
-      <c r="Y63" s="17" t="inlineStr">
-        <is>
-          <t>variant: transpose_free</t>
-        </is>
-      </c>
-      <c r="Z63" s="17">
-        <f>Z11+Z40+2*(SUM(T41:T42))+SUM(T43:T44)+T45+Z56+SUM(T57:T61)</f>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>match readout (dual-softmax)</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>multiply</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="n">
+        <v>513</v>
+      </c>
+      <c r="D62" s="11" t="n">
+        <v>513</v>
+      </c>
+      <c r="E62" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" s="13" t="n">
+        <v>513</v>
+      </c>
+      <c r="M62" s="13" t="n">
+        <v>513</v>
+      </c>
+      <c r="N62" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" s="3">
+        <f>C62*D62/1024</f>
+        <v/>
+      </c>
+      <c r="P62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" s="3">
+        <f>L62*M62/1024</f>
+        <v/>
+      </c>
+      <c r="S62" s="3">
+        <f>C62*D62/128</f>
+        <v/>
+      </c>
+      <c r="T62" s="3">
+        <f>(S62/$Y$2)/1000</f>
+        <v/>
+      </c>
+      <c r="U62" s="26">
+        <f>((O62*8*1024)/$T62)/1000</f>
+        <v/>
+      </c>
+      <c r="V62" s="26">
+        <f>((P62*8*1024)/$T62)/1000</f>
+        <v/>
+      </c>
+      <c r="W62" s="26">
+        <f>((Q62*8*1024)/$T62)/1000</f>
+        <v/>
+      </c>
+      <c r="X62" s="26">
+        <f>((R62*8*1024)/$T62)/1000</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
+          <t>GRAND TOTAL [us]</t>
+        </is>
+      </c>
+      <c r="Y64" s="17" t="inlineStr">
+        <is>
+          <t>variant: transpose_free</t>
+        </is>
+      </c>
+      <c r="Z64" s="17">
+        <f>Z11+Z40+2*(SUM(T41:T42))+SUM(T43:T44)+T45+Z57+SUM(T58:T62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
           <t>FPS (image pair)</t>
         </is>
       </c>
-      <c r="Y64" s="17" t="inlineStr">
+      <c r="Y65" s="17" t="inlineStr">
         <is>
           <t>frames / sec -&gt;</t>
         </is>
       </c>
-      <c r="Z64" s="17">
-        <f>1000000/Z63</f>
+      <c r="Z65" s="17">
+        <f>1000000/Z64</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="AA21:AA30"/>
-    <mergeCell ref="AA12:AA40"/>
-    <mergeCell ref="AA3:AA11"/>
-    <mergeCell ref="AA41:AA61"/>
-    <mergeCell ref="AA47:AA56"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -32519,7 +32292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA62"/>
+  <dimension ref="A1:Z62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36.109375" customWidth="1" min="1" max="1"/>
@@ -32855,11 +32628,6 @@
         <f>((R3*8*1024)/$T3)/1000</f>
         <v/>
       </c>
-      <c r="AA3" s="44" t="inlineStr">
-        <is>
-          <t>Keypoint Encoder (x2 images)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -32946,7 +32714,6 @@
         <f>((R4*8*1024)/$T4)/1000</f>
         <v/>
       </c>
-      <c r="AA4" s="47" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -33033,7 +32800,6 @@
         <f>((R5*8*1024)/$T5)/1000</f>
         <v/>
       </c>
-      <c r="AA5" s="47" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -33120,7 +32886,6 @@
         <f>((R6*8*1024)/$T6)/1000</f>
         <v/>
       </c>
-      <c r="AA6" s="47" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -33207,7 +32972,6 @@
         <f>((R7*8*1024)/$T7)/1000</f>
         <v/>
       </c>
-      <c r="AA7" s="47" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -33294,7 +33058,6 @@
         <f>((R8*8*1024)/$T8)/1000</f>
         <v/>
       </c>
-      <c r="AA8" s="47" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -33381,7 +33144,6 @@
         <f>((R9*8*1024)/$T9)/1000</f>
         <v/>
       </c>
-      <c r="AA9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -33468,7 +33230,6 @@
         <f>((R10*8*1024)/$T10)/1000</f>
         <v/>
       </c>
-      <c r="AA10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -33564,7 +33325,6 @@
         <f>2*(SUM(T3:T11))</f>
         <v/>
       </c>
-      <c r="AA11" s="48" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -33651,11 +33411,6 @@
         <f>((R12*8*1024)/$T12)/1000</f>
         <v/>
       </c>
-      <c r="AA12" s="44" t="inlineStr">
-        <is>
-          <t>Attentional GNN block (x36=18 layers x2 img)</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -33742,7 +33497,6 @@
         <f>((R13*8*1024)/$T13)/1000</f>
         <v/>
       </c>
-      <c r="AA13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -33829,7 +33583,6 @@
         <f>((R14*8*1024)/$T14)/1000</f>
         <v/>
       </c>
-      <c r="AA14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -33916,7 +33669,6 @@
         <f>((R15*8*1024)/$T15)/1000</f>
         <v/>
       </c>
-      <c r="AA15" s="47" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -34003,7 +33755,6 @@
         <f>((R16*8*1024)/$T16)/1000</f>
         <v/>
       </c>
-      <c r="AA16" s="47" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -34090,7 +33841,6 @@
         <f>((R17*8*1024)/$T17)/1000</f>
         <v/>
       </c>
-      <c r="AA17" s="47" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -34173,7 +33923,6 @@
       <c r="X18" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="47" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -34256,7 +34005,6 @@
       <c r="X19" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA19" s="47" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -34339,7 +34087,6 @@
       <c r="X20" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA20" s="47" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -34426,7 +34173,6 @@
         <f>((R21*8*1024)/$T21)/1000</f>
         <v/>
       </c>
-      <c r="AA21" s="47" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -34513,7 +34259,6 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
-      <c r="AA22" s="47" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -34600,7 +34345,6 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
-      <c r="AA23" s="47" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -34687,7 +34431,6 @@
         <f>((R24*8*1024)/$T24)/1000</f>
         <v/>
       </c>
-      <c r="AA24" s="47" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -34774,7 +34517,6 @@
         <f>((R25*8*1024)/$T25)/1000</f>
         <v/>
       </c>
-      <c r="AA25" s="47" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -34861,7 +34603,6 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
-      <c r="AA26" s="47" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -34948,7 +34689,6 @@
         <f>((R27*8*1024)/$T27)/1000</f>
         <v/>
       </c>
-      <c r="AA27" s="47" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -35035,7 +34775,6 @@
         <f>((R28*8*1024)/$T28)/1000</f>
         <v/>
       </c>
-      <c r="AA28" s="47" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -35122,7 +34861,6 @@
         <f>((R29*8*1024)/$T29)/1000</f>
         <v/>
       </c>
-      <c r="AA29" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -35209,7 +34947,6 @@
         <f>((R30*8*1024)/$T30)/1000</f>
         <v/>
       </c>
-      <c r="AA30" s="47" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -35301,7 +35038,6 @@
         <f>4*(SUM(T21:T30))</f>
         <v/>
       </c>
-      <c r="AA31" s="47" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -35388,7 +35124,6 @@
         <f>((R32*8*1024)/$T32)/1000</f>
         <v/>
       </c>
-      <c r="AA32" s="47" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -35475,7 +35210,6 @@
         <f>((R33*8*1024)/$T33)/1000</f>
         <v/>
       </c>
-      <c r="AA33" s="47" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -35562,7 +35296,6 @@
         <f>((R34*8*1024)/$T34)/1000</f>
         <v/>
       </c>
-      <c r="AA34" s="47" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -35649,7 +35382,6 @@
         <f>((R35*8*1024)/$T35)/1000</f>
         <v/>
       </c>
-      <c r="AA35" s="47" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -35736,7 +35468,6 @@
         <f>((R36*8*1024)/$T36)/1000</f>
         <v/>
       </c>
-      <c r="AA36" s="47" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -35823,7 +35554,6 @@
         <f>((R37*8*1024)/$T37)/1000</f>
         <v/>
       </c>
-      <c r="AA37" s="47" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -35910,7 +35640,6 @@
         <f>((R38*8*1024)/$T38)/1000</f>
         <v/>
       </c>
-      <c r="AA38" s="47" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -35997,7 +35726,6 @@
         <f>((R39*8*1024)/$T39)/1000</f>
         <v/>
       </c>
-      <c r="AA39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -36093,7 +35821,6 @@
         <f>36*(SUM(T12:T40)+3*(SUM(T21:T30)))</f>
         <v/>
       </c>
-      <c r="AA40" s="48" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -36180,11 +35907,6 @@
         <f>((R41*8*1024)/$T41)/1000</f>
         <v/>
       </c>
-      <c r="AA41" s="44" t="inlineStr">
-        <is>
-          <t>Matching</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -36271,7 +35993,6 @@
         <f>((R42*8*1024)/$T42)/1000</f>
         <v/>
       </c>
-      <c r="AA42" s="47" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -36358,7 +36079,6 @@
         <f>((R43*8*1024)/$T43)/1000</f>
         <v/>
       </c>
-      <c r="AA43" s="47" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -36445,7 +36165,6 @@
         <f>((R44*8*1024)/$T44)/1000</f>
         <v/>
       </c>
-      <c r="AA44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -36532,7 +36251,6 @@
         <f>((R45*8*1024)/$T45)/1000</f>
         <v/>
       </c>
-      <c r="AA45" s="47" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -36615,7 +36333,6 @@
       <c r="X46" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="AA46" s="47" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -36702,7 +36419,6 @@
         <f>((R47*8*1024)/$T47)/1000</f>
         <v/>
       </c>
-      <c r="AA47" s="47" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -36789,7 +36505,6 @@
         <f>((R48*8*1024)/$T48)/1000</f>
         <v/>
       </c>
-      <c r="AA48" s="47" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -36876,7 +36591,6 @@
         <f>((R49*8*1024)/$T49)/1000</f>
         <v/>
       </c>
-      <c r="AA49" s="47" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -36963,7 +36677,6 @@
         <f>((R50*8*1024)/$T50)/1000</f>
         <v/>
       </c>
-      <c r="AA50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -37050,7 +36763,6 @@
         <f>((R51*8*1024)/$T51)/1000</f>
         <v/>
       </c>
-      <c r="AA51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -37137,7 +36849,6 @@
         <f>((R52*8*1024)/$T52)/1000</f>
         <v/>
       </c>
-      <c r="AA52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -37224,7 +36935,6 @@
         <f>((R53*8*1024)/$T53)/1000</f>
         <v/>
       </c>
-      <c r="AA53" s="47" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -37311,7 +37021,6 @@
         <f>((R54*8*1024)/$T54)/1000</f>
         <v/>
       </c>
-      <c r="AA54" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -37398,7 +37107,6 @@
         <f>((R55*8*1024)/$T55)/1000</f>
         <v/>
       </c>
-      <c r="AA55" s="47" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -37485,7 +37193,6 @@
         <f>((R56*8*1024)/$T56)/1000</f>
         <v/>
       </c>
-      <c r="AA56" s="47" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -37581,7 +37288,6 @@
         <f>100*(SUM(T47:T57))</f>
         <v/>
       </c>
-      <c r="AA57" s="47" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -37668,7 +37374,6 @@
         <f>((R58*8*1024)/$T58)/1000</f>
         <v/>
       </c>
-      <c r="AA58" s="47" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -37755,7 +37460,6 @@
         <f>((R59*8*1024)/$T59)/1000</f>
         <v/>
       </c>
-      <c r="AA59" s="48" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -37790,13 +37494,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="AA47:AA57"/>
-    <mergeCell ref="AA21:AA30"/>
-    <mergeCell ref="AA12:AA40"/>
-    <mergeCell ref="AA3:AA11"/>
-    <mergeCell ref="AA41:AA59"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -37807,7 +37504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z28"/>
+  <dimension ref="A1:Z29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36.109375" customWidth="1" min="1" max="1"/>
@@ -38049,7 +37746,9 @@
       <c r="X2" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y2" t="inlineStr"/>
+      <c r="Y2" t="n">
+        <v>1</v>
+      </c>
       <c r="Z2" t="n">
         <v>8</v>
       </c>
@@ -38512,7 +38211,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C8" s="11" t="n">
@@ -38602,7 +38301,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
@@ -38692,7 +38391,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
@@ -38782,7 +38481,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
@@ -38867,7 +38566,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>scale 1/sqrt(d)</t>
+          <t>scale</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -39052,7 +38751,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C14" s="11" t="n">
@@ -39137,12 +38836,12 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>out proj D-&gt;D</t>
+          <t>out proj</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
@@ -39322,7 +39021,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
@@ -39502,7 +39201,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C19" s="11" t="n">
@@ -39682,7 +39381,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
@@ -39772,7 +39471,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>MAC matmul</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
@@ -39848,12 +39547,11 @@
         <f>((R22*8*1024)/$T22)/1000</f>
         <v/>
       </c>
-      <c r="Y22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>scale 1/sqrt(d)</t>
+          <t>scale</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -39934,7 +39632,6 @@
         <f>((R23*8*1024)/$T23)/1000</f>
         <v/>
       </c>
-      <c r="Y23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -39944,7 +39641,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>sum,scale</t>
+          <t>sum+scale</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
@@ -40034,7 +39731,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>ACC.MAX,scale</t>
+          <t>ACC.MAX+scale</t>
         </is>
       </c>
       <c r="C25" s="11" t="n">
@@ -40200,37 +39897,36 @@
         <f>((R26*8*1024)/$T26)/1000</f>
         <v/>
       </c>
-      <c r="Y26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL [us] (measured)</t>
-        </is>
-      </c>
-      <c r="Y27" s="17" t="inlineStr">
-        <is>
-          <t>measured emulator cycles -&gt;</t>
-        </is>
-      </c>
-      <c r="Z27" s="17">
-        <f>SUM(T2:T26)</f>
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
+          <t>GRAND TOTAL [us] (measured)</t>
+        </is>
+      </c>
+      <c r="Y28" s="17" t="inlineStr">
+        <is>
+          <t>measured emulator cycles -&gt;</t>
+        </is>
+      </c>
+      <c r="Z28" s="17">
+        <f>SUM(T2:T26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
           <t>FPS (image pair)</t>
         </is>
       </c>
-      <c r="Y28" s="17" t="inlineStr">
+      <c r="Y29" s="17" t="inlineStr">
         <is>
           <t>frames / sec -&gt;</t>
         </is>
       </c>
-      <c r="Z28" s="17">
-        <f>1000000/Z27</f>
+      <c r="Z29" s="17">
+        <f>1000000/Z28</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: use softmax_mt for SuperGlue attention softmax (N=512)
measure_kernels.py: add measure_softmax_mt() and include 'softmax_mt_512': 88
in rates(). build_sg_excel.py: new 'sm_mt' opcyc kind = d * softmax_mt_512;
the attention-softmax row in the measured sheet now uses one softmax_mt call
per row instead of 4 independent softmax128 tiles (the previous model was
incorrect -- N=512 softmax needs cross-tile reduction, not 4 independent
128-softmaxes). All six sheets still PASS Python<->XLS cross-validation;
measured total 1.655 M us -> 0.60 FPS.

https://claude.ai/code/session_01Wj1AhpfDtCg3YHVUGoUUbF
</commit_message>
<xml_diff>
--- a/IPU_2_SuperGlue.xlsx
+++ b/IPU_2_SuperGlue.xlsx
@@ -59666,12 +59666,12 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>softmax</t>
+          <t>softmax (multi-tile)</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>max,exp2,sum,mul</t>
+          <t>softmax_mt.asm</t>
         </is>
       </c>
       <c r="C36" s="11" t="n">
@@ -59725,7 +59725,7 @@
         <v/>
       </c>
       <c r="S36" s="3" t="n">
-        <v>5603328</v>
+        <v>6488064</v>
       </c>
       <c r="T36" s="3">
         <f>(S36/$Y$2)/1000</f>

</xml_diff>

<commit_message>
Revert: don't apply softmax_mt to SuperGlue attention in the measured sheet
User clarified softmax_mt is intended for SuperPoint, not SuperGlue. Restore
the SuperGlue attention softmax row to the previous single-tile 'sm' model.
softmax_mt.asm itself stays as a validated kernel for future use. All six
sheets still PASS Python<->XLS validation; measured total back to 1.654 M us.

https://claude.ai/code/session_01Wj1AhpfDtCg3YHVUGoUUbF
</commit_message>
<xml_diff>
--- a/IPU_2_SuperGlue.xlsx
+++ b/IPU_2_SuperGlue.xlsx
@@ -59666,12 +59666,12 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>softmax (multi-tile)</t>
+          <t>softmax</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>softmax_mt.asm</t>
+          <t>max,exp2,sum,mul</t>
         </is>
       </c>
       <c r="C36" s="11" t="n">
@@ -59725,7 +59725,7 @@
         <v/>
       </c>
       <c r="S36" s="3" t="n">
-        <v>6488064</v>
+        <v>5603328</v>
       </c>
       <c r="T36" s="3">
         <f>(S36/$Y$2)/1000</f>

</xml_diff>

<commit_message>
Excel: detector softmax(65) uses softmax_mt.asm (single-tile, 42 cyc)
measure_kernels.py: measure softmax_mt at both ntiles=1 (N<=128 -> 42 cyc) and
ntiles=4 (N=512 -> 88 cyc); rates() returns softmax_mt_1, softmax_mt_4.
build_sg_excel.py: 'sm_mt' opcyc selects the right rate by tiles(c). SuperPoint
detector softmax(65 channels per pixel) row now routes to softmax_mt.asm at
42 cyc/softmax. Measured total 1.654 -> 1.655 M us (+221 us). All six sheets
PASS Python<->XLS validation.

https://claude.ai/code/session_01Wj1AhpfDtCg3YHVUGoUUbF
</commit_message>
<xml_diff>
--- a/IPU_2_SuperGlue.xlsx
+++ b/IPU_2_SuperGlue.xlsx
@@ -57796,7 +57796,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>softmax</t>
+          <t>softmax_mt.asm</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
@@ -57850,7 +57850,7 @@
         <v/>
       </c>
       <c r="S15" s="3" t="n">
-        <v>182400</v>
+        <v>403200</v>
       </c>
       <c r="T15" s="3">
         <f>(S15/$Y$2)/1000</f>

</xml_diff>